<commit_message>
Client Web Page Folder Structure Updated
</commit_message>
<xml_diff>
--- a/Files/Excel Template.xlsx
+++ b/Files/Excel Template.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t xml:space="preserve">S_no</t>
   </si>
@@ -43,19 +43,22 @@
     <t xml:space="preserve">Department</t>
   </si>
   <si>
+    <t xml:space="preserve">FC001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VinoPriya K</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Faculty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AIDS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Admin001</t>
+  </si>
+  <si>
     <t xml:space="preserve">sarankiruthik</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-+</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Faculty</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AIDS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Admin001</t>
   </si>
   <si>
     <t xml:space="preserve">sknexus.exp@gmail.com</t>
@@ -81,7 +84,6 @@
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -104,7 +106,6 @@
       <color theme="0"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <charset val="1"/>
     </font>
     <font>
       <u val="single"/>
@@ -112,7 +113,6 @@
       <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -166,20 +166,24 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -303,14 +307,14 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204" pitchFamily="0" charset="1"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="0" charset="1"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme>
@@ -318,67 +322,25 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:tint val="67000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:tint val="73000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:tint val="81000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
-        </a:gradFill>
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:shade val="78000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
-        </a:gradFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
         <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
+          <a:miter/>
         </a:ln>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
+          <a:miter/>
         </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
+          <a:miter/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
@@ -397,35 +359,11 @@
           <a:schemeClr val="phClr"/>
         </a:solidFill>
         <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
-        </a:gradFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
@@ -441,79 +379,77 @@
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="24.27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="32.63"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="10.82"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="19.91"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="14.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="32.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="10.82"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="2" width="19.91"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="1" t="n">
-        <v>620822243093</v>
-      </c>
-      <c r="C2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="C2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="0" t="n">
+      <c r="D2" s="5"/>
+      <c r="E2" s="2" t="n">
         <v>8072682003</v>
       </c>
-      <c r="F2" s="0" t="s">
+      <c r="F2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="0" t="s">
+      <c r="G2" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2" t="n">
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="0" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3" s="4" t="s">
+      <c r="C3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E3" s="0" t="n">
+      <c r="D3" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="2" t="n">
         <v>9487605484</v>
       </c>
-      <c r="F3" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="G3" s="0" t="s">
+      <c r="F3" s="2" t="s">
         <v>14</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>